<commit_message>
update commodity units for whole energy system model
</commit_message>
<xml_diff>
--- a/input_excels/vt_DE_helper.xlsx
+++ b/input_excels/vt_DE_helper.xlsx
@@ -11722,17 +11722,22 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_pow</t>
+          <t>sec_elec_a</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11771,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -11778,58 +11783,68 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_a</t>
+          <t>emi_co2_neg_fuel_cc_x2x</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>emi_co2_neg_fuel_cc_pow</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>exo_sec_elec_f</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pri_wind_energy_e</t>
+          <t>iip_chemi_mtg_mtk_h2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -11846,17 +11861,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pri_geoth_heat</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -11868,24 +11878,29 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>pri_geoth_heat_g</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_b</t>
+          <t>exo_sec_elec_d</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -11895,7 +11910,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -11907,7 +11922,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>pri_wind_energy</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -11919,39 +11934,29 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>exo_sec_elec_e</t>
+          <t>pri_wind_energy_e</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iip_chemi_methanol</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Mt</t>
+          <t>sec_saving</t>
         </is>
       </c>
     </row>
@@ -11963,7 +11968,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>pri_wind_energy</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -11980,17 +11985,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sec_elec_b</t>
+          <t>pri_marine_d</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12002,24 +12002,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>sec_heating_oil</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>iip_chemi_lpg</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12031,12 +12031,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>iip_steel_blafu_gas_in</t>
+          <t>sec_elec_ind</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12048,7 +12053,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -12065,7 +12070,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>pri_solar_radiation_g</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -12082,17 +12087,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_elec_e</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12104,34 +12104,29 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>iip_auto_space_heat</t>
+          <t>iip_steel_coke_oven_gas_in</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>iip_chemi_nh3</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12143,7 +12138,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -12160,19 +12155,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_saving</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>exo_sec_elec_c</t>
+          <t>pri_geoth_heat</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -12182,24 +12177,29 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ELC</t>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>emi_co2_neg_proc_cc_ind</t>
+          <t>exo_sec_elec_g</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12211,12 +12211,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
+          <t>pri_geoth_heat_e</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12228,7 +12233,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>pri_solar_radiation_f</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -12240,17 +12245,17 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_ind</t>
+          <t>iip_chemi_methanol</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
@@ -12262,17 +12267,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_c</t>
+          <t>pri_wind_energy_a</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12284,34 +12284,29 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_e</t>
+          <t>iip_steel_blafu_gas_in</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_x2x</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12323,34 +12318,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>pri_wind_energy_a</t>
+          <t>pri_geoth_heat_d</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>exo_sec_elec_d</t>
+          <t>pri_marine_g</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12362,7 +12357,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>pri_marine_g</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -12374,22 +12369,17 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>exo_sec_elec_b</t>
+          <t>iip_chemi_nh3</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
@@ -12401,7 +12391,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>pri_bio_wood</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -12418,7 +12408,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>pri_wind_energy_d</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -12430,17 +12420,22 @@
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>pri_geoth_heat_b</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12452,17 +12447,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sec_elec_d</t>
+          <t>pri_marine_c</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12474,46 +12464,56 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>iip_chemi_steam</t>
+          <t>sec_elec_e</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>iip_chemi_biomethanol</t>
+          <t>pri_solar_radiation_a</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>exo_sec_elec_b</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12525,7 +12525,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_g</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -12535,24 +12535,24 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>iip_chemi_mtg_mtk_h2</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>pri_envir_heat</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12564,34 +12564,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>sec_elec_f</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>exo_sec_elec</t>
+          <t>pri_marine_e</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12603,7 +12603,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>pri_marine_f</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -12620,68 +12620,73 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>iip_auto_space_heat</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>emi_co2_stored</t>
+          <t>pri_wind_energy_b</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Kt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>iip_chemi_nh3_h2</t>
+          <t>sec_elec_distr</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sec_elec_g</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -12693,7 +12698,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_a</t>
+          <t>iip_elec</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -12703,36 +12708,36 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>pri_wind_energy_d</t>
+          <t>iip_chemi_biomethanol</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>iip_chemi_meoh_h2</t>
+          <t>sec_kerosene_fos_orig</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -12749,7 +12754,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>pri_marine_c</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -12766,51 +12771,41 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sec_elec_c</t>
+          <t>pri_marine_b</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>exo_sec_elec_a</t>
+          <t>iip_steel_coke_oven_gas</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>iip_chemi_heavy_fuel_oil</t>
+          <t>sec_biomethanol_orig</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -12822,29 +12817,34 @@
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>pri_wind_energy_c</t>
+          <t>exo_sec_elec</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_f</t>
+          <t>exo_sec_elec_a</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -12854,7 +12854,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_g</t>
+          <t>pri_solar_radiation_d</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -12883,36 +12883,46 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>sec_heating_oil</t>
+          <t>sec_gasoline_fos_orig</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>iip_chemi_lpg</t>
+          <t>pri_geoth_heat_c</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>pri_wind_energy_g</t>
+          <t>iip_chemi_biomass</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -12924,12 +12934,12 @@
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>iip_chemi_biomass</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -12946,7 +12956,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>iip_steel_coke_oven_gas_in</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -12963,12 +12973,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>sec_biomethanol_orig</t>
+          <t>pri_geoth_heat_f</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12980,7 +12995,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>sec_natural_gas_syn</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12992,7 +13012,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>pri_marine_a</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -13009,7 +13029,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_f</t>
+          <t>pri_marine</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -13021,17 +13041,17 @@
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -13043,7 +13063,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>pri_marine_a</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -13060,7 +13080,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_b</t>
+          <t>iip_chemi_steam</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -13072,12 +13092,12 @@
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>iip_chemi_methane</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -13094,7 +13114,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_d</t>
+          <t>pri_wind_energy_c</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -13111,7 +13131,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -13128,12 +13148,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>pri_solar_radiation</t>
+          <t>sec_elec_g</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13145,12 +13170,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>pri_wind_energy_f</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>sec_diesel</t>
         </is>
       </c>
     </row>
@@ -13162,7 +13182,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>pri_marine_e</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -13174,34 +13194,29 @@
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>sec_elec_f</t>
+          <t>iip_chemi_meoh_h2</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>exo_sec_elec_g</t>
+          <t>pri_geoth_heat_a</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -13211,7 +13226,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>ELC</t>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -13223,7 +13238,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -13240,7 +13255,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>sec_elec_c</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13252,17 +13277,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_d</t>
+          <t>pri_solar_radiation_e</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -13274,12 +13294,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>iip_steel_blafu_gas</t>
+          <t>sec_elec_b</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13291,17 +13316,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>sec_elec_distr</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13313,46 +13333,46 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>pri_wind_energy_f</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>sec_biokerosene_orig</t>
+          <t>exo_sec_elec_c</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>pri_wind_energy_b</t>
+          <t>iip_chemi_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -13369,7 +13389,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>sec_methane</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -13381,17 +13401,17 @@
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>pri_marine_b</t>
+          <t>emi_co2_neg_proc_cc_ind</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13423,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>iip_chemi_naphtha</t>
+          <t>iip_chemi_nh3_h2</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -13420,12 +13440,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>iip_steel_coke_oven_gas</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>pri_crude_oil</t>
         </is>
       </c>
     </row>
@@ -13437,12 +13452,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_c</t>
+          <t>sec_elec_d</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13454,12 +13474,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>pri_marine</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
     </row>
@@ -13471,7 +13486,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
+          <t>pri_solar_radiation_b</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -13488,7 +13503,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_e</t>
+          <t>pri_solar_radiation_c</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -13505,17 +13520,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>iip_elec</t>
+          <t>pri_solar_radiation</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13527,7 +13537,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_biokerosene_orig</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -13539,22 +13549,17 @@
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>exo_sec_elec_f</t>
+          <t>iip_steel_blafu_gas</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13583,7 +13588,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>pri_bio_wood</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -13600,7 +13605,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>pri_marine_f</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -13612,12 +13617,12 @@
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>pri_marine_d</t>
+          <t>iip_chemi_methane</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -13629,39 +13634,34 @@
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>sec_elec_a</t>
+          <t>iip_chemi_naphtha</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>pri_envir_heat</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>emi_co2_stored</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -13673,46 +13673,46 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>sec_elec_ind</t>
+          <t>pri_wind_energy_g</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>exo_sec_elec_e</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
+          <t>emi_co2_neg_fuel_cc_ind</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -13813,12 +13813,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Activity Unit</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>PJ</t>
+          <t>Capacity Unit</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -13828,12 +13828,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>Operational Commodity Group</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>Vintage Tracking</t>
         </is>
       </c>
     </row>

</xml_diff>